<commit_message>
feat(parsers): nrb-bfi-monthly-xlsx v0.3.0 — C7 sector-loan extraction
Extends the BFI monthly parser to also parse sheet C7 (Statement of
Loans & Advances by sector). C7 provides productive-sector and structural
credit data that closes the SME/productive-sector data gap: agriculture,
electricity, tourism, construction, wholesale, finance/insurance, consumption,
the sectorwise total, and deprived-sector loans — all by bank class.

Files with no C7 sheet (14-sheet format, pre-Chaitra 2079) return
status='partial' with a PageLayoutChanged error; C5 data is unaffected.

22/22 tests pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scrapers/nrb_bfi/tests/fixtures/Asoj_2082_Publish.xlsx
+++ b/scrapers/nrb_bfi/tests/fixtures/Asoj_2082_Publish.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C5" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C6" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C7" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -674,4 +675,189 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B7:AE15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Agricultural and Forest Related</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>5000.5</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4000.5</v>
+      </c>
+      <c r="W7" t="n">
+        <v>700.5</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>300.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Electricity,Gas and Water</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>5001.5</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4001.5</v>
+      </c>
+      <c r="W8" t="n">
+        <v>701.5</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>301.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tourism Service**</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>5002.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>4002.5</v>
+      </c>
+      <c r="W9" t="n">
+        <v>702.5</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>302.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>5003.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>4003.5</v>
+      </c>
+      <c r="W10" t="n">
+        <v>703.5</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>303.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wholesaler &amp; Retailer</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>5004.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4004.5</v>
+      </c>
+      <c r="W11" t="n">
+        <v>704.5</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>304.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Finance, Insurance and Real Estate</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>5005.5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4005.5</v>
+      </c>
+      <c r="W12" t="n">
+        <v>705.5</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>305.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Consumption Loans</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>5006.5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4006.5</v>
+      </c>
+      <c r="W13" t="n">
+        <v>706.5</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>306.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>5007.5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>4007.5</v>
+      </c>
+      <c r="W14" t="n">
+        <v>707.5</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>307.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Deprived Sector Loan</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>5008.5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>4008.5</v>
+      </c>
+      <c r="W15" t="n">
+        <v>708.5</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>308.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>